<commit_message>
PPC report: apply CRM check (Rita Williams lost to competitor, Susan Delgado reopened)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JRjkL7ZhPzEbkxd56QrxaQ
</commit_message>
<xml_diff>
--- a/reports/Juan_PPC_Lead_Report.xlsx
+++ b/reports/Juan_PPC_Lead_Report.xlsx
@@ -1021,7 +1021,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C27" s="6">
         <f>B27/SUM($B$26:$B$36)</f>
@@ -1091,7 +1091,7 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C32" s="6">
         <f>B32/SUM($B$26:$B$36)</f>
@@ -1274,7 +1274,7 @@
         </is>
       </c>
       <c r="B46" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="47">
@@ -74813,12 +74813,17 @@
       </c>
       <c r="F1723" t="inlineStr">
         <is>
-          <t>Under Contract</t>
+          <t>Offer Rejected</t>
         </is>
       </c>
       <c r="G1723" t="inlineStr">
         <is>
           <t>7 Cancelled Contract</t>
+        </is>
+      </c>
+      <c r="I1723" t="inlineStr">
+        <is>
+          <t>CRM: Lost – sold to competitor</t>
         </is>
       </c>
       <c r="J1723" t="inlineStr">
@@ -75035,7 +75040,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Rita Williams</t>
+          <t>Rita Williams (CRM: Lost/Dead · 9 Lost · Sold to Competitor)</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -75050,7 +75055,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Under Contract</t>
+          <t>Lost – sold to competitor</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -75203,7 +75208,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Susan Delgado</t>
+          <t>Susan Delgado (CRM: reopened, Active · 2 Follow Up / Unresponsive)</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">

</xml_diff>